<commit_message>
Populate fixed packaging fields in every import SKU
</commit_message>
<xml_diff>
--- a/desktop/assets/运动短袖短裤套装.xlsx
+++ b/desktop/assets/运动短袖短裤套装.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:Q6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -477,6 +477,31 @@
           <t>SKU属性</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>外包装形状</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>外包装类型</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>外包装图片</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>是否定制品</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>是否敏感属性</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -484,7 +509,6 @@
           <t>女装运动圆领高腰T恤短裤套装</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
           <t>混合色</t>
@@ -515,7 +539,6 @@
           <t>200.0</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>29046</t>
@@ -529,6 +552,31 @@
       <c r="L2" t="inlineStr">
         <is>
           <t>[{"specId":21263,"parentSpecName":"颜色","specName":"混合色","parentSpecId":1001},{"specId":10004,"parentSpecName":"尺码","specName":"S","parentSpecId":3001}]</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>长方体</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>软包装+软物</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>https://img.cdnfe.com/product/open/ad7a1f90a1b744c08ed8a93b5c0fd982-goods.jpeg</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>否</t>
         </is>
       </c>
     </row>
@@ -538,7 +586,6 @@
           <t>女装运动圆领高腰T恤短裤套装</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>混合色</t>
@@ -569,7 +616,6 @@
           <t>200.0</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
           <t>29046</t>
@@ -583,6 +629,31 @@
       <c r="L3" t="inlineStr">
         <is>
           <t>[{"specId":21263,"parentSpecName":"颜色","specName":"混合色","parentSpecId":1001},{"specId":9005,"parentSpecName":"尺码","specName":"M","parentSpecId":3001}]</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>长方体</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>软包装+软物</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>https://img.cdnfe.com/product/open/ad7a1f90a1b744c08ed8a93b5c0fd982-goods.jpeg</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>否</t>
         </is>
       </c>
     </row>
@@ -592,7 +663,6 @@
           <t>女装运动圆领高腰T恤短裤套装</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>混合色</t>
@@ -623,7 +693,6 @@
           <t>200.0</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
           <t>29046</t>
@@ -637,6 +706,31 @@
       <c r="L4" t="inlineStr">
         <is>
           <t>[{"specId":21263,"parentSpecName":"颜色","specName":"混合色","parentSpecId":1001},{"specId":11002,"parentSpecName":"尺码","specName":"L","parentSpecId":3001}]</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>长方体</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>软包装+软物</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>https://img.cdnfe.com/product/open/ad7a1f90a1b744c08ed8a93b5c0fd982-goods.jpeg</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>否</t>
         </is>
       </c>
     </row>
@@ -646,7 +740,6 @@
           <t>女装运动圆领高腰T恤短裤套装</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>混合色</t>
@@ -677,7 +770,6 @@
           <t>200.0</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
           <t>29046</t>
@@ -691,6 +783,31 @@
       <c r="L5" t="inlineStr">
         <is>
           <t>[{"specId":21263,"parentSpecName":"颜色","specName":"混合色","parentSpecId":1001},{"specId":12003,"parentSpecName":"尺码","specName":"XL","parentSpecId":3001}]</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>长方体</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>软包装+软物</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>https://img.cdnfe.com/product/open/ad7a1f90a1b744c08ed8a93b5c0fd982-goods.jpeg</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>否</t>
         </is>
       </c>
     </row>
@@ -700,7 +817,6 @@
           <t>女装运动圆领高腰T恤短裤套装</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>混合色</t>
@@ -731,7 +847,6 @@
           <t>200.0</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
           <t>29046</t>
@@ -745,6 +860,31 @@
       <c r="L6" t="inlineStr">
         <is>
           <t>[{"specId":21263,"parentSpecName":"颜色","specName":"混合色","parentSpecId":1001},{"specId":8002,"parentSpecName":"尺码","specName":"XXL","parentSpecId":3001}]</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>长方体</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>软包装+软物</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>https://img.cdnfe.com/product/open/ad7a1f90a1b744c08ed8a93b5c0fd982-goods.jpeg</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>否</t>
         </is>
       </c>
     </row>

</xml_diff>